<commit_message>
Retro #2 (ADR-034): human_minutes đo thời gian người; reviewer độc lập TRƯỚC khi duyệt
- Schema log + build_report(+excel): tính tiết kiệm theo human_minutes, không dùng wall-clock
- seed_demo_data: thêm human_minutes
- playbooks/pr-review-loop.md: reviewer độc lập (agent context mới) chạy TRƯỚC PO người duyệt
- Rút từ lần review độc lập thật tìm ra 6 lỗi bị bỏ sót ở WeatherApp

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>57.0%</t>
+          <t>91.0%</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>0.62</v>
+        <v>0.92</v>
       </c>
       <c r="E2" t="n">
         <v>8</v>
@@ -711,7 +711,7 @@
         <v>30</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>0.52</v>
+        <v>0.9</v>
       </c>
       <c r="E3" t="n">
         <v>9</v>
@@ -1001,7 +1001,7 @@
         <v>57</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>0.61</v>
+        <v>0.91</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1061,7 +1061,7 @@
         <v>91</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>0.62</v>
+        <v>0.92</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1125,7 +1125,7 @@
         <v>47</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>0.62</v>
+        <v>0.89</v>
       </c>
       <c r="I7" t="n">
         <v>15</v>
@@ -1185,7 +1185,7 @@
         <v>234</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>0.62</v>
+        <v>0.92</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1249,7 +1249,7 @@
         <v>68</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>0.62</v>
+        <v>0.93</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1313,7 +1313,7 @@
         <v>117</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>0.62</v>
+        <v>0.92</v>
       </c>
       <c r="I10" t="n">
         <v>30</v>
@@ -1373,7 +1373,7 @@
         <v>78</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>0.62</v>
+        <v>0.92</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1433,7 +1433,7 @@
         <v>116</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>0.53</v>
+        <v>0.91</v>
       </c>
       <c r="I12" t="n">
         <v>60</v>
@@ -1497,7 +1497,7 @@
         <v>252</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.52</v>
+        <v>0.9</v>
       </c>
       <c r="I13" t="n">
         <v>240</v>
@@ -1561,7 +1561,7 @@
         <v>84</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>0.52</v>
+        <v>0.9</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1621,7 +1621,7 @@
         <v>158</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.53</v>
+        <v>0.91</v>
       </c>
       <c r="I15" t="n">
         <v>120</v>
@@ -1685,7 +1685,7 @@
         <v>126</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>0.52</v>
+        <v>0.9</v>
       </c>
       <c r="I16" t="n">
         <v>30</v>
@@ -1749,7 +1749,7 @@
         <v>101</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.52</v>
+        <v>0.9</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
@@ -1813,7 +1813,7 @@
         <v>200</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>0.52</v>
+        <v>0.9</v>
       </c>
       <c r="I18" t="n">
         <v>45</v>

</xml_diff>